<commit_message>
Added new RDF data schemes and visual schemes for education-table03-07, fixed XLSX spreadsheets for education-table04-07
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/education-table04.xlsx
+++ b/sources/table_normalization/xlsx/education-table04.xlsx
@@ -484,7 +484,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="27">
+  <fills count="28">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -638,6 +638,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1749,65 +1755,6 @@
     <xf numFmtId="0" fontId="4" fillId="26" borderId="27" xfId="468" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="1" xfId="473" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="1" xfId="473" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="1" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="472" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="472" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="472" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="472" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" xfId="467" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="467" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="469" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="2" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="473" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="7" xfId="473" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1836,6 +1783,65 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="26" xfId="473" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" xfId="467" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="467" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="469" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="2" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="1" xfId="473" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="472" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="472" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="472" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="26" xfId="472" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="473" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="1" xfId="473" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="543">
     <cellStyle name="20% - Accent1 2" xfId="2"/>
@@ -2795,24 +2801,24 @@
       <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1">
-      <c r="A3" s="48"/>
-      <c r="B3" s="47"/>
-      <c r="C3" s="49" t="s">
+      <c r="A3" s="47"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="49"/>
-      <c r="J3" s="49"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="61" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
@@ -2821,22 +2827,22 @@
       <c r="D4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="50" t="s">
+      <c r="E4" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="51"/>
-      <c r="G4" s="50" t="s">
+      <c r="F4" s="73"/>
+      <c r="G4" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="52"/>
-      <c r="I4" s="53" t="s">
+      <c r="H4" s="74"/>
+      <c r="I4" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="52"/>
+      <c r="J4" s="74"/>
     </row>
     <row r="5" spans="1:10" ht="45" customHeight="1">
-      <c r="A5" s="59"/>
-      <c r="B5" s="59"/>
+      <c r="A5" s="62"/>
+      <c r="B5" s="62"/>
       <c r="C5" s="42" t="s">
         <v>9</v>
       </c>
@@ -2863,39 +2869,39 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="15" customHeight="1">
-      <c r="A6" s="60" t="s">
+      <c r="A6" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="68" t="s">
+      <c r="B6" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="69">
+      <c r="C6" s="48">
         <v>1312100</v>
       </c>
-      <c r="D6" s="70">
+      <c r="D6" s="49">
         <v>1449800</v>
       </c>
-      <c r="E6" s="71">
+      <c r="E6" s="50">
         <v>1430600</v>
       </c>
-      <c r="F6" s="72">
+      <c r="F6" s="51">
         <v>-1.2999999999999999E-2</v>
       </c>
-      <c r="G6" s="71">
+      <c r="G6" s="50">
         <v>1471300</v>
       </c>
-      <c r="H6" s="72">
+      <c r="H6" s="51">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="I6" s="73">
+      <c r="I6" s="52">
         <v>1538300</v>
       </c>
-      <c r="J6" s="72">
+      <c r="J6" s="51">
         <v>4.5999999999999999E-2</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1">
-      <c r="A7" s="61"/>
+      <c r="A7" s="64"/>
       <c r="B7" s="9" t="s">
         <v>15</v>
       </c>
@@ -2925,7 +2931,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1">
-      <c r="A8" s="61"/>
+      <c r="A8" s="64"/>
       <c r="B8" s="12" t="s">
         <v>16</v>
       </c>
@@ -2955,7 +2961,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="15" customHeight="1">
-      <c r="A9" s="61"/>
+      <c r="A9" s="64"/>
       <c r="B9" s="12" t="s">
         <v>17</v>
       </c>
@@ -2985,7 +2991,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="15" customHeight="1">
-      <c r="A10" s="61"/>
+      <c r="A10" s="64"/>
       <c r="B10" s="15" t="s">
         <v>18</v>
       </c>
@@ -3015,7 +3021,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="15" customHeight="1">
-      <c r="A11" s="61"/>
+      <c r="A11" s="64"/>
       <c r="B11" s="17" t="s">
         <v>19</v>
       </c>
@@ -3045,7 +3051,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="15" customHeight="1">
-      <c r="A12" s="61"/>
+      <c r="A12" s="64"/>
       <c r="B12" s="12" t="s">
         <v>16</v>
       </c>
@@ -3075,7 +3081,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1">
-      <c r="A13" s="61"/>
+      <c r="A13" s="64"/>
       <c r="B13" s="12" t="s">
         <v>17</v>
       </c>
@@ -3105,7 +3111,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="15" customHeight="1">
-      <c r="A14" s="61"/>
+      <c r="A14" s="64"/>
       <c r="B14" s="15" t="s">
         <v>18</v>
       </c>
@@ -3135,7 +3141,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
-      <c r="A15" s="61"/>
+      <c r="A15" s="64"/>
       <c r="B15" s="18" t="s">
         <v>20</v>
       </c>
@@ -3165,7 +3171,7 @@
       </c>
     </row>
     <row r="16" spans="1:10" ht="15" customHeight="1">
-      <c r="A16" s="61"/>
+      <c r="A16" s="64"/>
       <c r="B16" s="12" t="s">
         <v>16</v>
       </c>
@@ -3195,7 +3201,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1">
-      <c r="A17" s="61"/>
+      <c r="A17" s="64"/>
       <c r="B17" s="12" t="s">
         <v>17</v>
       </c>
@@ -3225,7 +3231,7 @@
       </c>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1">
-      <c r="A18" s="62"/>
+      <c r="A18" s="65"/>
       <c r="B18" s="15" t="s">
         <v>18</v>
       </c>
@@ -3255,39 +3261,39 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1">
-      <c r="A19" s="60" t="s">
+      <c r="A19" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="68" t="s">
+      <c r="B19" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="74">
+      <c r="C19" s="53">
         <v>812600</v>
       </c>
-      <c r="D19" s="75">
+      <c r="D19" s="54">
         <v>965900</v>
       </c>
-      <c r="E19" s="76">
+      <c r="E19" s="55">
         <v>952400</v>
       </c>
-      <c r="F19" s="72">
+      <c r="F19" s="51">
         <v>-1.4E-2</v>
       </c>
-      <c r="G19" s="76">
+      <c r="G19" s="55">
         <v>910200</v>
       </c>
-      <c r="H19" s="72">
+      <c r="H19" s="51">
         <v>-4.3999999999999997E-2</v>
       </c>
-      <c r="I19" s="77">
+      <c r="I19" s="56">
         <v>921700</v>
       </c>
-      <c r="J19" s="72">
+      <c r="J19" s="51">
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1">
-      <c r="A20" s="61"/>
+      <c r="A20" s="64"/>
       <c r="B20" s="9" t="s">
         <v>15</v>
       </c>
@@ -3317,7 +3323,7 @@
       </c>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1">
-      <c r="A21" s="61"/>
+      <c r="A21" s="64"/>
       <c r="B21" s="12" t="s">
         <v>16</v>
       </c>
@@ -3347,7 +3353,7 @@
       </c>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1">
-      <c r="A22" s="61"/>
+      <c r="A22" s="64"/>
       <c r="B22" s="12" t="s">
         <v>17</v>
       </c>
@@ -3377,7 +3383,7 @@
       </c>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1">
-      <c r="A23" s="61"/>
+      <c r="A23" s="64"/>
       <c r="B23" s="15" t="s">
         <v>18</v>
       </c>
@@ -3407,7 +3413,7 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1">
-      <c r="A24" s="61"/>
+      <c r="A24" s="64"/>
       <c r="B24" s="17" t="s">
         <v>19</v>
       </c>
@@ -3437,7 +3443,7 @@
       </c>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1">
-      <c r="A25" s="61"/>
+      <c r="A25" s="64"/>
       <c r="B25" s="12" t="s">
         <v>16</v>
       </c>
@@ -3467,7 +3473,7 @@
       </c>
     </row>
     <row r="26" spans="1:10" ht="15" customHeight="1">
-      <c r="A26" s="61"/>
+      <c r="A26" s="64"/>
       <c r="B26" s="12" t="s">
         <v>17</v>
       </c>
@@ -3497,7 +3503,7 @@
       </c>
     </row>
     <row r="27" spans="1:10" ht="15" customHeight="1">
-      <c r="A27" s="61"/>
+      <c r="A27" s="64"/>
       <c r="B27" s="15" t="s">
         <v>18</v>
       </c>
@@ -3527,7 +3533,7 @@
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" customHeight="1">
-      <c r="A28" s="61"/>
+      <c r="A28" s="64"/>
       <c r="B28" s="18" t="s">
         <v>20</v>
       </c>
@@ -3557,7 +3563,7 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="15" customHeight="1">
-      <c r="A29" s="61"/>
+      <c r="A29" s="64"/>
       <c r="B29" s="12" t="s">
         <v>16</v>
       </c>
@@ -3587,7 +3593,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" ht="15" customHeight="1">
-      <c r="A30" s="61"/>
+      <c r="A30" s="64"/>
       <c r="B30" s="12" t="s">
         <v>17</v>
       </c>
@@ -3617,7 +3623,7 @@
       </c>
     </row>
     <row r="31" spans="1:10" ht="15" customHeight="1">
-      <c r="A31" s="62"/>
+      <c r="A31" s="65"/>
       <c r="B31" s="15" t="s">
         <v>18</v>
       </c>
@@ -3657,135 +3663,140 @@
       <c r="F32" s="4"/>
     </row>
     <row r="33" spans="1:10" ht="30" customHeight="1">
-      <c r="A33" s="54" t="s">
+      <c r="A33" s="57" t="s">
         <v>24</v>
       </c>
-      <c r="B33" s="54"/>
-      <c r="C33" s="54"/>
-      <c r="D33" s="54"/>
-      <c r="E33" s="54"/>
-      <c r="F33" s="54"/>
-      <c r="G33" s="54"/>
-      <c r="H33" s="54"/>
-      <c r="I33" s="54"/>
-      <c r="J33" s="54"/>
+      <c r="B33" s="57"/>
+      <c r="C33" s="57"/>
+      <c r="D33" s="57"/>
+      <c r="E33" s="57"/>
+      <c r="F33" s="57"/>
+      <c r="G33" s="57"/>
+      <c r="H33" s="57"/>
+      <c r="I33" s="57"/>
+      <c r="J33" s="57"/>
     </row>
     <row r="34" spans="1:10" ht="15" customHeight="1">
-      <c r="A34" s="63" t="s">
+      <c r="A34" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="B34" s="63"/>
-      <c r="C34" s="63"/>
-      <c r="D34" s="63"/>
-      <c r="E34" s="63"/>
-      <c r="F34" s="63"/>
-      <c r="G34" s="63"/>
-      <c r="H34" s="63"/>
-      <c r="I34" s="63"/>
-      <c r="J34" s="63"/>
+      <c r="B34" s="66"/>
+      <c r="C34" s="66"/>
+      <c r="D34" s="66"/>
+      <c r="E34" s="66"/>
+      <c r="F34" s="66"/>
+      <c r="G34" s="66"/>
+      <c r="H34" s="66"/>
+      <c r="I34" s="66"/>
+      <c r="J34" s="66"/>
     </row>
     <row r="35" spans="1:10" ht="30" customHeight="1">
-      <c r="A35" s="64" t="s">
+      <c r="A35" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="B35" s="64"/>
-      <c r="C35" s="64"/>
-      <c r="D35" s="64"/>
-      <c r="E35" s="64"/>
-      <c r="F35" s="64"/>
-      <c r="G35" s="64"/>
-      <c r="H35" s="64"/>
-      <c r="I35" s="64"/>
-      <c r="J35" s="64"/>
+      <c r="B35" s="67"/>
+      <c r="C35" s="67"/>
+      <c r="D35" s="67"/>
+      <c r="E35" s="67"/>
+      <c r="F35" s="67"/>
+      <c r="G35" s="67"/>
+      <c r="H35" s="67"/>
+      <c r="I35" s="67"/>
+      <c r="J35" s="67"/>
     </row>
     <row r="36" spans="1:10" ht="15" customHeight="1">
-      <c r="A36" s="65" t="s">
+      <c r="A36" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="B36" s="65"/>
-      <c r="C36" s="65"/>
-      <c r="D36" s="65"/>
-      <c r="E36" s="65"/>
-      <c r="F36" s="65"/>
-      <c r="G36" s="65"/>
-      <c r="H36" s="65"/>
-      <c r="I36" s="65"/>
-      <c r="J36" s="65"/>
+      <c r="B36" s="68"/>
+      <c r="C36" s="68"/>
+      <c r="D36" s="68"/>
+      <c r="E36" s="68"/>
+      <c r="F36" s="68"/>
+      <c r="G36" s="68"/>
+      <c r="H36" s="68"/>
+      <c r="I36" s="68"/>
+      <c r="J36" s="68"/>
     </row>
     <row r="37" spans="1:10" ht="30" customHeight="1">
-      <c r="A37" s="66" t="s">
+      <c r="A37" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="B37" s="66"/>
-      <c r="C37" s="66"/>
-      <c r="D37" s="66"/>
-      <c r="E37" s="66"/>
-      <c r="F37" s="66"/>
-      <c r="G37" s="66"/>
-      <c r="H37" s="66"/>
-      <c r="I37" s="66"/>
-      <c r="J37" s="66"/>
+      <c r="B37" s="69"/>
+      <c r="C37" s="69"/>
+      <c r="D37" s="69"/>
+      <c r="E37" s="69"/>
+      <c r="F37" s="69"/>
+      <c r="G37" s="69"/>
+      <c r="H37" s="69"/>
+      <c r="I37" s="69"/>
+      <c r="J37" s="69"/>
     </row>
     <row r="38" spans="1:10" ht="15" customHeight="1">
-      <c r="A38" s="67" t="s">
+      <c r="A38" s="70" t="s">
         <v>29</v>
       </c>
-      <c r="B38" s="67"/>
-      <c r="C38" s="67"/>
-      <c r="D38" s="67"/>
-      <c r="E38" s="67"/>
-      <c r="F38" s="67"/>
-      <c r="G38" s="67"/>
-      <c r="H38" s="67"/>
-      <c r="I38" s="67"/>
-      <c r="J38" s="67"/>
+      <c r="B38" s="70"/>
+      <c r="C38" s="70"/>
+      <c r="D38" s="70"/>
+      <c r="E38" s="70"/>
+      <c r="F38" s="70"/>
+      <c r="G38" s="70"/>
+      <c r="H38" s="70"/>
+      <c r="I38" s="70"/>
+      <c r="J38" s="70"/>
     </row>
     <row r="39" spans="1:10">
-      <c r="A39" s="54" t="s">
+      <c r="A39" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="B39" s="54"/>
-      <c r="C39" s="54"/>
-      <c r="D39" s="54"/>
-      <c r="E39" s="54"/>
-      <c r="F39" s="54"/>
+      <c r="B39" s="57"/>
+      <c r="C39" s="57"/>
+      <c r="D39" s="57"/>
+      <c r="E39" s="57"/>
+      <c r="F39" s="57"/>
       <c r="G39" s="39"/>
       <c r="H39" s="39"/>
       <c r="I39" s="40"/>
       <c r="J39" s="40"/>
     </row>
     <row r="40" spans="1:10">
-      <c r="A40" s="55"/>
-      <c r="B40" s="55"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="55"/>
-      <c r="F40" s="55"/>
+      <c r="A40" s="58"/>
+      <c r="B40" s="58"/>
+      <c r="C40" s="58"/>
+      <c r="D40" s="58"/>
+      <c r="E40" s="58"/>
+      <c r="F40" s="58"/>
       <c r="G40" s="34"/>
       <c r="H40" s="34"/>
     </row>
     <row r="41" spans="1:10">
-      <c r="A41" s="56"/>
-      <c r="B41" s="55"/>
-      <c r="C41" s="55"/>
-      <c r="D41" s="55"/>
-      <c r="E41" s="55"/>
-      <c r="F41" s="55"/>
+      <c r="A41" s="59"/>
+      <c r="B41" s="58"/>
+      <c r="C41" s="58"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="58"/>
       <c r="G41" s="34"/>
       <c r="H41" s="34"/>
     </row>
     <row r="42" spans="1:10">
-      <c r="A42" s="57"/>
-      <c r="B42" s="57"/>
-      <c r="C42" s="57"/>
-      <c r="D42" s="57"/>
-      <c r="E42" s="57"/>
-      <c r="F42" s="57"/>
+      <c r="A42" s="60"/>
+      <c r="B42" s="60"/>
+      <c r="C42" s="60"/>
+      <c r="D42" s="60"/>
+      <c r="E42" s="60"/>
+      <c r="F42" s="60"/>
       <c r="G42" s="34"/>
       <c r="H42" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C3:J3"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="A33:J33"/>
     <mergeCell ref="A39:F39"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="A41:F41"/>
@@ -3799,11 +3810,6 @@
     <mergeCell ref="A36:J36"/>
     <mergeCell ref="A37:J37"/>
     <mergeCell ref="A38:J38"/>
-    <mergeCell ref="C3:J3"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A33:J33"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A34" r:id="rId1"/>

</xml_diff>